<commit_message>
Modela o que tem dentro do Armário 3 e põe o número do móvel nos códigos
- Botão "Fechar armário" (e Esc) fecha as portas e volta a câmera para o laboratório.
- Armário 3 ganha o que aparece na foto: caixas das estações Yaxun, cesto de solda,
  terceira mão, organizadores e as duas pilhas de caixinhas. Cada caixinha é um
  compartimento clicável (P3C-1, P3D-4…), com a etiqueta lida na foto.
- Os códigos levam o número do móvel: P3A a P3D no Armário 3, G6A a G6D no
  Gaveteiro 6, C12A a C12E na Maleta 12. O link fica #G6A ou #P3C-1.
- Clicar num compartimento com coisas dentro aproxima a câmera dele.
- A busca encontra também as etiquetas das caixinhas e o que está no modelo.
- Portas, gavetas e câmera animam pelo relógio, igual em qualquer taxa de quadros.
- Planilha modelo regenerada com os novos códigos e os itens do Armário 3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ferramentas/planilha_armarios_neon.xlsx
+++ b/ferramentas/planilha_armarios_neon.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Estoque'!$A$1:$L$1000</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Locais'!$A$1:$D$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Locais'!$A$1:$D$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -237,7 +237,7 @@
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2. Local no armário é o código do compartimento: G1 é a gaveta 1, P2 é a prateleira 2, P2A é o lado esquerdo da prateleira 2 e C1 é o compartimento 1 de uma caixa ou maleta.</t>
+          <t>2. Local no armário é o código do compartimento. Ele leva o número do móvel: P3A é a primeira prateleira do Armário 3, G6B é a segunda gaveta do Gaveteiro 6, C12A é o primeiro compartimento da Maleta 12 e P3C-1 é a caixinha 1 da P3C.</t>
         </is>
       </c>
     </row>
@@ -275,7 +275,7 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Gaveteiro 6  |  G1  |  Eletrônica  |  Conectores  |  XT60 fêmea  |  Amass, original  |  10  |  un  |  Novo  |  (vazio)  |  26/10/2026  |  (vazio)</t>
+          <t>Gaveteiro 6  |  G6A  |  Eletrônica  |  Conectores  |  XT60 fêmea  |  Amass, original  |  10  |  un  |  Novo  |  (vazio)  |  26/10/2026  |  (vazio)</t>
         </is>
       </c>
     </row>
@@ -334,7 +334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -421,7 +421,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>C1A</t>
+          <t>C12A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>C1B</t>
+          <t>C12B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>C1C</t>
+          <t>C12C</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>C1C</t>
+          <t>C12C</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>C1D</t>
+          <t>C12D</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C12E</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C12E</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C12E</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C12E</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -802,6 +802,689 @@
       <c r="L10" t="inlineStr">
         <is>
           <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>P3A</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Ferramentas</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Estação de retrabalho Yaxun</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Solda e ar quente, na caixa azul</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>P3A</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ferramentas</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Estação de retrabalho SMD Yaxun</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Ar quente, nas caixas pretas</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>P3B</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ferramentas</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Terceira mão com limpador de ponta</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Braços flexíveis e base com lã de latão</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>P3B</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Termo retrátil</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>No organizador transparente</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>P3B</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ferramentas</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Cesto de solda</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ferro de solda, alicates e chaves</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório. Veja o que tem dentro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>P3C-3</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Cola quente</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>P3C-6</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Conectores</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Terminais</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>P3C-10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Cabos</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>P3C-11</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Placas e controladores</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Arduino</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>P3C-12</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Cabo USB do Arduino</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>P3D-1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Fita crepe</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>rolo</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>P3D-2</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Protoboard</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>P3D-4</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Fita isolante</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>rolo</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>P3D-8</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Baterias</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Pilhas</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>P3D-10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>P3D-11</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>P3D-12</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>P3D-13</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>P3D</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Borrifador</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Líquido transparente</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório. Confira o que tem dentro.</t>
         </is>
       </c>
     </row>
@@ -834,7 +1517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -922,7 +1605,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>P2A</t>
+          <t>P1C</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -944,7 +1627,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>P2B</t>
+          <t>P1D</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -966,7 +1649,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>P1A</t>
+          <t>P2A</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -988,7 +1671,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>P1B</t>
+          <t>P2B</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -1010,7 +1693,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>P2A</t>
+          <t>P2C</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -1032,7 +1715,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>P2B</t>
+          <t>P2D</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -1054,7 +1737,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>P1A</t>
+          <t>P3A</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -1076,7 +1759,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>P1B</t>
+          <t>P3B</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1098,7 +1781,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>P2A</t>
+          <t>P3C</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1120,743 +1803,1359 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>P2B</t>
+          <t>P3C-1</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, esquerda · caixinha 1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Armário 4</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Maletas de ferramentas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>P1A</t>
+          <t>P3C-2</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, esquerda</t>
+          <t>Prateleira 2, esquerda · caixinha 2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Armário 4</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Maletas de ferramentas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>P1B</t>
+          <t>P3C-3</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, direita</t>
+          <t>Prateleira 2, esquerda · caixinha 3 (Cola quente)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Armário 4</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Maletas de ferramentas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>P2A</t>
+          <t>P3C-4</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 2, esquerda · caixinha 4</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Armário 4</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Maletas de ferramentas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>P2B</t>
+          <t>P3C-5</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, esquerda · caixinha 5</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Armário 5</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Kits de componentes</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>P1A</t>
+          <t>P3C-6</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, esquerda</t>
+          <t>Prateleira 2, esquerda · caixinha 6 (Terminais)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Armário 5</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Kits de componentes</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>P1B</t>
+          <t>P3C-7</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, direita</t>
+          <t>Prateleira 2, esquerda · caixinha 7</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Armário 5</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Kits de componentes</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>P2A</t>
+          <t>P3C-8</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 2, esquerda · caixinha 8</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Armário 5</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Kits de componentes</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>P2B</t>
+          <t>P3C-9</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, esquerda · caixinha 9</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 6</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Bancada branca</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>P3C-10</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 1</t>
+          <t>Prateleira 2, esquerda · caixinha 10 (Cabos)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 6</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Bancada branca</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>P3C-11</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 2</t>
+          <t>Prateleira 2, esquerda · caixinha 11 (Arduino)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 6</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Bancada branca</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>P3C-12</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 3</t>
+          <t>Prateleira 2, esquerda · caixinha 12 (Cabos USB do Arduino)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 6</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Bancada branca</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>P3C-13</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 4</t>
+          <t>Prateleira 2, esquerda · caixinha 13</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Armário 7</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Ferramentas e tintas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>P1A</t>
+          <t>P3C-14</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, esquerda</t>
+          <t>Prateleira 2, esquerda · caixinha 14</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Armário 7</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Ferramentas e tintas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>P1B</t>
+          <t>P3C-15</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, direita</t>
+          <t>Prateleira 2, esquerda · caixinha 15</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Armário 7</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Ferramentas e tintas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>P2A</t>
+          <t>P3D</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 2, direita</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Armário 7</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Ferramentas e tintas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>P2B</t>
+          <t>P3D-1</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, direita · caixinha 1 (Fita crepe)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 8</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Volante, bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>P3D-2</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 1</t>
+          <t>Prateleira 2, direita · caixinha 2 (Protoboard)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 8</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Volante, bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>P3D-3</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 2</t>
+          <t>Prateleira 2, direita · caixinha 3</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 8</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Volante, bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>P3D-4</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 3</t>
+          <t>Prateleira 2, direita · caixinha 4 (Fita isolante)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Caixa 9</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Caixa preta, no chão</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>P3D-5</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Dentro da caixa</t>
+          <t>Prateleira 2, direita · caixinha 5</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 10</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>P3D-6</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 1</t>
+          <t>Prateleira 2, direita · caixinha 6</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 10</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>P3D-7</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 2</t>
+          <t>Prateleira 2, direita · caixinha 7</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 10</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>P3D-8</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 3</t>
+          <t>Prateleira 2, direita · caixinha 8 (Pilhas)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 10</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>P3D-9</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 4</t>
+          <t>Prateleira 2, direita · caixinha 9</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Armário 11</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>P1A</t>
+          <t>P3D-10</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, esquerda</t>
+          <t>Prateleira 2, direita · caixinha 10 (Jumpers)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>Armário 11</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>P1B</t>
+          <t>P3D-11</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, direita</t>
+          <t>Prateleira 2, direita · caixinha 11 (Jumpers)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>Armário 11</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>P2A</t>
+          <t>P3D-12</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 2, direita · caixinha 12 (Jumpers)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>Armário 11</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>P2B</t>
+          <t>P3D-13</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, direita · caixinha 13 (Jumpers)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>Maleta 12</t>
+          <t>Armário 4</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Motores e rádio</t>
+          <t>Maletas de ferramentas</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>C1A</t>
+          <t>P4A</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Bandeja, divisão A</t>
+          <t>Prateleira 1, esquerda</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Maleta 12</t>
+          <t>Armário 4</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Motores e rádio</t>
+          <t>Maletas de ferramentas</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>C1B</t>
+          <t>P4B</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Bandeja, divisão B</t>
+          <t>Prateleira 1, direita</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Maleta 12</t>
+          <t>Armário 4</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Motores e rádio</t>
+          <t>Maletas de ferramentas</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>C1C</t>
+          <t>P4C</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Bandeja, divisão C</t>
+          <t>Prateleira 2, esquerda</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Maleta 12</t>
+          <t>Armário 4</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Motores e rádio</t>
+          <t>Maletas de ferramentas</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>C1D</t>
+          <t>P4D</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Bandeja, divisão D</t>
+          <t>Prateleira 2, direita</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
+          <t>Armário 5</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Kits de componentes</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>P5A</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 1, esquerda</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Armário 5</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Kits de componentes</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>P5B</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 1, direita</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Armário 5</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Kits de componentes</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>P5C</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 2, esquerda</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Armário 5</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Kits de componentes</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>P5D</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 2, direita</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 6</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Bancada branca</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>G6A</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 6</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Bancada branca</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>G6B</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 6</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Bancada branca</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>G6C</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 6</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Bancada branca</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>G6D</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Armário 7</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Ferramentas e tintas</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>P7A</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 1, esquerda</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>Armário 7</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Ferramentas e tintas</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>P7B</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 1, direita</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Armário 7</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Ferramentas e tintas</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>P7C</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 2, esquerda</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Armário 7</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Ferramentas e tintas</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>P7D</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 2, direita</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 8</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Volante, bancada preta</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>G8A</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 8</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Volante, bancada preta</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>G8B</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 8</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Volante, bancada preta</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>G8C</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>Caixa 9</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Caixa preta, no chão</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Dentro da caixa</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 10</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Bancada preta</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>G10A</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 10</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Bancada preta</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>G10B</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 10</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Bancada preta</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>G10C</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>Gaveteiro 10</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Bancada preta</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>G10D</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Gaveta 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>Armário 11</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Bancada preta</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>P11A</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 1, esquerda</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>Armário 11</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Bancada preta</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>P11B</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 1, direita</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>Armário 11</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Bancada preta</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>P11C</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 2, esquerda</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>Armário 11</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Bancada preta</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>P11D</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Prateleira 2, direita</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
           <t>Maleta 12</t>
         </is>
       </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="B70" s="7" t="inlineStr">
         <is>
           <t>Motores e rádio</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>C12A</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja, divisão 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>Maleta 12</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Motores e rádio</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>C12B</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja, divisão 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>Maleta 12</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Motores e rádio</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>C12C</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja, divisão 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>Maleta 12</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Motores e rádio</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>C12D</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja, divisão 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>Maleta 12</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Motores e rádio</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>C12E</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
         <is>
           <t>Fundo da maleta</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D46"/>
+  <autoFilter ref="A1:D74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cesto de solda abre as ferramentas em cima da bancada
- O cesto rosa do Armário 3 vira o compartimento P3B-1. Ao clicar nele, as 18
  coisas da foto de 27/10/2026 aparecem na bancada embaixo do armário, com nome,
  e a câmera olha a bancada de cima. Clicar de novo guarda tudo.
- Novas formas para o modelo: ferro de solda, suporte do ferro, alicates (corte,
  crimpador e desencapador), pinças no saquinho, carretel, escova e manta;
  cilindro com conta-gotas, tampa reta ou deitado.
- O painel lista o que está na bancada e a busca acha cada ferramenta.
- Rótulos da bancada não se cobrem: o que não acha espaço fica escondido.
- Planilha modelo com os 18 itens do cesto em P3B-1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ferramentas/planilha_armarios_neon.xlsx
+++ b/ferramentas/planilha_armarios_neon.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Estoque'!$A$1:$L$1000</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Locais'!$A$1:$D$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Locais'!$A$1:$D$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -334,7 +334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -985,7 +985,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>P3B</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1000,12 +1000,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Cesto de solda</t>
+          <t>Ferro de solda</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ferro de solda, alicates e chaves</t>
+          <t>Cabo amarelo e preto</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório. Veja o que tem dentro.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1030,22 +1030,40 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>P3C-3</t>
+          <t>P3B-1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cola quente</t>
+          <t>Ferro de solda Hikari</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Cabo branco</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1075,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>P3C-6</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1067,17 +1085,30 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Conectores</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Terminais</t>
+          <t>Suporte para ferro de solda Yaxun</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Azul, com bandeja para a esponja</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1120,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>P3C-10</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1099,17 +1130,30 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Cabos</t>
+          <t>Alicate de corte rente Hikari</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Cabo amarelo e preto</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1165,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>P3C-11</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1131,17 +1175,30 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Placas e controladores</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Arduino</t>
+          <t>Alicate de corte rente pequeno</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Cabo cinza</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1210,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>P3C-12</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1163,17 +1220,30 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Cabo USB do Arduino</t>
+          <t>Alicate crimpador de terminais</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Cabo vermelho e azul</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1185,27 +1255,40 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>P3D-1</t>
+          <t>P3B-1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fita crepe</t>
-        </is>
+          <t>Alicate desencapador automático</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Laranja e amarelo</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>rolo</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1300,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>P3D-2</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1227,13 +1310,21 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Protoboard</t>
-        </is>
+          <t>Alicate desencapador automático</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Vermelho e preto</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1242,7 +1333,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1345,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>P3D-4</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1264,22 +1355,30 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fita isolante</t>
-        </is>
+          <t>Pinça antiestática</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>No saquinho amarelo</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>rolo</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Confira quantas pinças tem no saquinho.</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1390,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>P3D-8</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1301,22 +1400,30 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Baterias</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pilhas</t>
-        </is>
+          <t>Jogo de pinças antiestáticas</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>6 pinças, pontas retas e curvas</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1435,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>P3D-10</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1338,17 +1445,30 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Jumpers</t>
+          <t>Estanho (fio de solda)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Carretel</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>rolo</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Parecem 2 carretéis empilhados.</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1480,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>P3D-11</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1370,17 +1490,30 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Jumpers</t>
+          <t>Pasta de solda Cobix</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Pote de 110 g</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1525,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>P3D-12</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1402,17 +1535,30 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Jumpers</t>
+          <t>Fluxo de solda líquido</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Frasco com bico; o rótulo começa com "Res"</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Leia o rótulo para confirmar o que é.</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1570,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>P3D-13</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1434,17 +1580,30 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Jumpers</t>
+          <t>Malha dessoldadora</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Carretel pequeno roxo</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1456,22 +1615,27 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>P3D</t>
+          <t>P3B-1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Borrifador</t>
+          <t>Sugador de solda</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Líquido transparente</t>
+          <t>Azul</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -1483,6 +1647,602 @@
         </is>
       </c>
       <c r="L29" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>P3B-1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Ferramentas</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Escova pequena de limpeza</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Cerdas pretas</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>P3B-1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Ferramentas</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Manta de silicone para solda</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Azul, com divisórias</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Confira se ela fica guardada no cesto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>P3B-1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Peça preta de plástico</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Retangular, com uma janela no meio</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Não deu para saber o que é pela foto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>P3C-3</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Cola quente</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>P3C-6</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Conectores</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Terminais</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>P3C-10</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Cabos</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>P3C-11</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Placas e controladores</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Arduino</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>P3C-12</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Cabo USB do Arduino</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>P3D-1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Fita crepe</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>rolo</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>P3D-2</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Protoboard</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>P3D-4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Fita isolante</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>rolo</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>P3D-8</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Baterias</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Pilhas</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>P3D-10</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>P3D-11</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>P3D-12</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>P3D-13</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>P3D</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Consumíveis</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Borrifador</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Líquido transparente</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
         <is>
           <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório. Confira o que tem dentro.</t>
         </is>
@@ -1517,7 +2277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1781,12 +2541,12 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>P3C</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 1, direita · cesto de solda</t>
         </is>
       </c>
     </row>
@@ -1803,12 +2563,12 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>P3C-1</t>
+          <t>P3C</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 1</t>
+          <t>Prateleira 2, esquerda</t>
         </is>
       </c>
     </row>
@@ -1825,12 +2585,12 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>P3C-2</t>
+          <t>P3C-1</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 2</t>
+          <t>Prateleira 2, esquerda · caixinha 1</t>
         </is>
       </c>
     </row>
@@ -1847,12 +2607,12 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>P3C-3</t>
+          <t>P3C-2</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 3 (Cola quente)</t>
+          <t>Prateleira 2, esquerda · caixinha 2</t>
         </is>
       </c>
     </row>
@@ -1869,12 +2629,12 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>P3C-4</t>
+          <t>P3C-3</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 4</t>
+          <t>Prateleira 2, esquerda · caixinha 3 (Cola quente)</t>
         </is>
       </c>
     </row>
@@ -1891,12 +2651,12 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>P3C-5</t>
+          <t>P3C-4</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 5</t>
+          <t>Prateleira 2, esquerda · caixinha 4</t>
         </is>
       </c>
     </row>
@@ -1913,12 +2673,12 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>P3C-6</t>
+          <t>P3C-5</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 6 (Terminais)</t>
+          <t>Prateleira 2, esquerda · caixinha 5</t>
         </is>
       </c>
     </row>
@@ -1935,12 +2695,12 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>P3C-7</t>
+          <t>P3C-6</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 7</t>
+          <t>Prateleira 2, esquerda · caixinha 6 (Terminais)</t>
         </is>
       </c>
     </row>
@@ -1957,12 +2717,12 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>P3C-8</t>
+          <t>P3C-7</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 8</t>
+          <t>Prateleira 2, esquerda · caixinha 7</t>
         </is>
       </c>
     </row>
@@ -1979,12 +2739,12 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>P3C-9</t>
+          <t>P3C-8</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 9</t>
+          <t>Prateleira 2, esquerda · caixinha 8</t>
         </is>
       </c>
     </row>
@@ -2001,12 +2761,12 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>P3C-10</t>
+          <t>P3C-9</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 10 (Cabos)</t>
+          <t>Prateleira 2, esquerda · caixinha 9</t>
         </is>
       </c>
     </row>
@@ -2023,12 +2783,12 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>P3C-11</t>
+          <t>P3C-10</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 11 (Arduino)</t>
+          <t>Prateleira 2, esquerda · caixinha 10 (Cabos)</t>
         </is>
       </c>
     </row>
@@ -2045,12 +2805,12 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>P3C-12</t>
+          <t>P3C-11</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 12 (Cabos USB do Arduino)</t>
+          <t>Prateleira 2, esquerda · caixinha 11 (Arduino)</t>
         </is>
       </c>
     </row>
@@ -2067,12 +2827,12 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>P3C-13</t>
+          <t>P3C-12</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 13</t>
+          <t>Prateleira 2, esquerda · caixinha 12 (Cabos USB do Arduino)</t>
         </is>
       </c>
     </row>
@@ -2089,12 +2849,12 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>P3C-14</t>
+          <t>P3C-13</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 14</t>
+          <t>Prateleira 2, esquerda · caixinha 13</t>
         </is>
       </c>
     </row>
@@ -2111,12 +2871,12 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>P3C-15</t>
+          <t>P3C-14</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda · caixinha 15</t>
+          <t>Prateleira 2, esquerda · caixinha 14</t>
         </is>
       </c>
     </row>
@@ -2133,12 +2893,12 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>P3D</t>
+          <t>P3C-15</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, esquerda · caixinha 15</t>
         </is>
       </c>
     </row>
@@ -2155,12 +2915,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>P3D-1</t>
+          <t>P3D</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 1 (Fita crepe)</t>
+          <t>Prateleira 2, direita</t>
         </is>
       </c>
     </row>
@@ -2177,12 +2937,12 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>P3D-2</t>
+          <t>P3D-1</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 2 (Protoboard)</t>
+          <t>Prateleira 2, direita · caixinha 1 (Fita crepe)</t>
         </is>
       </c>
     </row>
@@ -2199,12 +2959,12 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>P3D-3</t>
+          <t>P3D-2</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 3</t>
+          <t>Prateleira 2, direita · caixinha 2 (Protoboard)</t>
         </is>
       </c>
     </row>
@@ -2221,12 +2981,12 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>P3D-4</t>
+          <t>P3D-3</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 4 (Fita isolante)</t>
+          <t>Prateleira 2, direita · caixinha 3</t>
         </is>
       </c>
     </row>
@@ -2243,12 +3003,12 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>P3D-5</t>
+          <t>P3D-4</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 5</t>
+          <t>Prateleira 2, direita · caixinha 4 (Fita isolante)</t>
         </is>
       </c>
     </row>
@@ -2265,12 +3025,12 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>P3D-6</t>
+          <t>P3D-5</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 6</t>
+          <t>Prateleira 2, direita · caixinha 5</t>
         </is>
       </c>
     </row>
@@ -2287,12 +3047,12 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>P3D-7</t>
+          <t>P3D-6</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 7</t>
+          <t>Prateleira 2, direita · caixinha 6</t>
         </is>
       </c>
     </row>
@@ -2309,12 +3069,12 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>P3D-8</t>
+          <t>P3D-7</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 8 (Pilhas)</t>
+          <t>Prateleira 2, direita · caixinha 7</t>
         </is>
       </c>
     </row>
@@ -2331,12 +3091,12 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>P3D-9</t>
+          <t>P3D-8</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 9</t>
+          <t>Prateleira 2, direita · caixinha 8 (Pilhas)</t>
         </is>
       </c>
     </row>
@@ -2353,12 +3113,12 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>P3D-10</t>
+          <t>P3D-9</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 10 (Jumpers)</t>
+          <t>Prateleira 2, direita · caixinha 9</t>
         </is>
       </c>
     </row>
@@ -2375,12 +3135,12 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>P3D-11</t>
+          <t>P3D-10</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 11 (Jumpers)</t>
+          <t>Prateleira 2, direita · caixinha 10 (Jumpers)</t>
         </is>
       </c>
     </row>
@@ -2397,12 +3157,12 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>P3D-12</t>
+          <t>P3D-11</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 12 (Jumpers)</t>
+          <t>Prateleira 2, direita · caixinha 11 (Jumpers)</t>
         </is>
       </c>
     </row>
@@ -2419,34 +3179,34 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>P3D-13</t>
+          <t>P3D-12</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita · caixinha 13 (Jumpers)</t>
+          <t>Prateleira 2, direita · caixinha 12 (Jumpers)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>Armário 4</t>
+          <t>Armário 3</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Maletas de ferramentas</t>
+          <t>Solda e componentes</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>P4A</t>
+          <t>P3D-13</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, esquerda</t>
+          <t>Prateleira 2, direita · caixinha 13 (Jumpers)</t>
         </is>
       </c>
     </row>
@@ -2463,12 +3223,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>P4B</t>
+          <t>P4A</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, direita</t>
+          <t>Prateleira 1, esquerda</t>
         </is>
       </c>
     </row>
@@ -2485,12 +3245,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>P4C</t>
+          <t>P4B</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 1, direita</t>
         </is>
       </c>
     </row>
@@ -2507,34 +3267,34 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>P4D</t>
+          <t>P4C</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, esquerda</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Armário 5</t>
+          <t>Armário 4</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Kits de componentes</t>
+          <t>Maletas de ferramentas</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>P5A</t>
+          <t>P4D</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, esquerda</t>
+          <t>Prateleira 2, direita</t>
         </is>
       </c>
     </row>
@@ -2551,12 +3311,12 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>P5B</t>
+          <t>P5A</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, direita</t>
+          <t>Prateleira 1, esquerda</t>
         </is>
       </c>
     </row>
@@ -2573,12 +3333,12 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>P5C</t>
+          <t>P5B</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 1, direita</t>
         </is>
       </c>
     </row>
@@ -2595,34 +3355,34 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>P5D</t>
+          <t>P5C</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, esquerda</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 6</t>
+          <t>Armário 5</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Bancada branca</t>
+          <t>Kits de componentes</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>G6A</t>
+          <t>P5D</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 1</t>
+          <t>Prateleira 2, direita</t>
         </is>
       </c>
     </row>
@@ -2639,12 +3399,12 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>G6B</t>
+          <t>G6A</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 2</t>
+          <t>Gaveta 1</t>
         </is>
       </c>
     </row>
@@ -2661,12 +3421,12 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>G6C</t>
+          <t>G6B</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 3</t>
+          <t>Gaveta 2</t>
         </is>
       </c>
     </row>
@@ -2683,34 +3443,34 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>G6D</t>
+          <t>G6C</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 4</t>
+          <t>Gaveta 3</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Armário 7</t>
+          <t>Gaveteiro 6</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Ferramentas e tintas</t>
+          <t>Bancada branca</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>P7A</t>
+          <t>G6D</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, esquerda</t>
+          <t>Gaveta 4</t>
         </is>
       </c>
     </row>
@@ -2727,12 +3487,12 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>P7B</t>
+          <t>P7A</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, direita</t>
+          <t>Prateleira 1, esquerda</t>
         </is>
       </c>
     </row>
@@ -2749,12 +3509,12 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>P7C</t>
+          <t>P7B</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 1, direita</t>
         </is>
       </c>
     </row>
@@ -2771,34 +3531,34 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>P7D</t>
+          <t>P7C</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, esquerda</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 8</t>
+          <t>Armário 7</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Volante, bancada preta</t>
+          <t>Ferramentas e tintas</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>G8A</t>
+          <t>P7D</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 1</t>
+          <t>Prateleira 2, direita</t>
         </is>
       </c>
     </row>
@@ -2815,12 +3575,12 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>G8B</t>
+          <t>G8A</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 2</t>
+          <t>Gaveta 1</t>
         </is>
       </c>
     </row>
@@ -2837,56 +3597,56 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>G8C</t>
+          <t>G8B</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 3</t>
+          <t>Gaveta 2</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Caixa 9</t>
+          <t>Gaveteiro 8</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Caixa preta, no chão</t>
+          <t>Volante, bancada preta</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>G8C</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Dentro da caixa</t>
+          <t>Gaveta 3</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Gaveteiro 10</t>
+          <t>Caixa 9</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Bancada preta</t>
+          <t>Caixa preta, no chão</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>G10A</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 1</t>
+          <t>Dentro da caixa</t>
         </is>
       </c>
     </row>
@@ -2903,12 +3663,12 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>G10B</t>
+          <t>G10A</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 2</t>
+          <t>Gaveta 1</t>
         </is>
       </c>
     </row>
@@ -2925,12 +3685,12 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>G10C</t>
+          <t>G10B</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 3</t>
+          <t>Gaveta 2</t>
         </is>
       </c>
     </row>
@@ -2947,19 +3707,19 @@
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>G10D</t>
+          <t>G10C</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Gaveta 4</t>
+          <t>Gaveta 3</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>Armário 11</t>
+          <t>Gaveteiro 10</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -2969,12 +3729,12 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>P11A</t>
+          <t>G10D</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, esquerda</t>
+          <t>Gaveta 4</t>
         </is>
       </c>
     </row>
@@ -2991,12 +3751,12 @@
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>P11B</t>
+          <t>P11A</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 1, direita</t>
+          <t>Prateleira 1, esquerda</t>
         </is>
       </c>
     </row>
@@ -3013,12 +3773,12 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>P11C</t>
+          <t>P11B</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, esquerda</t>
+          <t>Prateleira 1, direita</t>
         </is>
       </c>
     </row>
@@ -3035,34 +3795,34 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>P11D</t>
+          <t>P11C</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Prateleira 2, direita</t>
+          <t>Prateleira 2, esquerda</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>Maleta 12</t>
+          <t>Armário 11</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Motores e rádio</t>
+          <t>Bancada preta</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>C12A</t>
+          <t>P11D</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Bandeja, divisão 1</t>
+          <t>Prateleira 2, direita</t>
         </is>
       </c>
     </row>
@@ -3079,12 +3839,12 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>C12B</t>
+          <t>C12A</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Bandeja, divisão 2</t>
+          <t>Bandeja, divisão 1</t>
         </is>
       </c>
     </row>
@@ -3101,12 +3861,12 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>C12C</t>
+          <t>C12B</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>Bandeja, divisão 3</t>
+          <t>Bandeja, divisão 2</t>
         </is>
       </c>
     </row>
@@ -3123,12 +3883,12 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>C12D</t>
+          <t>C12C</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Bandeja, divisão 4</t>
+          <t>Bandeja, divisão 3</t>
         </is>
       </c>
     </row>
@@ -3145,17 +3905,39 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
+          <t>C12D</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja, divisão 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>Maleta 12</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Motores e rádio</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
           <t>C12E</t>
         </is>
       </c>
-      <c r="D74" s="7" t="inlineStr">
+      <c r="D75" s="7" t="inlineStr">
         <is>
           <t>Fundo da maleta</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D74"/>
+  <autoFilter ref="A1:D75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Garra azul de solda na P3B, com foto ao clicar
- Nova forma para o modelo: garra de solda de mesa, com morsa preta e três
  braços flexíveis de contas azuis, bicos laranja e garras jacaré. Fica no
  fundo da P3B do Armário 3, atrás do cesto de solda.
- Campo foto em laboratorio.js: ao clicar na coisa, a foto abre por cima do
  modelo. O painel da P3B também tem o botão, e a dica embaixo avisa.
- O volume invisível de uma prateleira não tapa mais o que está no fundo dela.
- Coluna Foto na aba Estoque: um item com foto ganha o botão Ver foto.
- Planilha modelo com a garra em P3B e a coluna Foto.
- A foto do produto fica em imagens/; a pasta fotos/ continua fora do site.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ferramentas/planilha_armarios_neon.xlsx
+++ b/ferramentas/planilha_armarios_neon.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Listas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Estoque'!$A$1:$L$1000</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Estoque'!$A$1:$M$1000</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Locais'!$A$1:$D$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -196,7 +196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B19"/>
+  <dimension ref="B1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -263,58 +263,65 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>5. A coluna Foto é opcional: um link de imagem (https://...) ou uma foto da pasta imagens do site (imagens/garra-azul-de-solda.jpg). No site, o item ganha o botão Ver foto.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Exemplo de linha na aba Estoque</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Gaveteiro 6  |  G6A  |  Eletrônica  |  Conectores  |  XT60 fêmea  |  Amass, original  |  10  |  un  |  Novo  |  (vazio)  |  26/10/2026  |  (vazio)</t>
-        </is>
-      </c>
-    </row>
     <row r="13">
-      <c r="B13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Gaveteiro 6  |  G6A  |  Eletrônica  |  Conectores  |  XT60 fêmea  |  Amass, original  |  10  |  un  |  Novo  |  (vazio)  |  26/10/2026  |  (vazio)  |  (vazio)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Os móveis do modelo</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Os móveis, as medidas e as gavetas de cada um ficam no próprio site, no arquivo laboratorio.js, e não nesta planilha.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Se um móvel mudar de lugar ou ganhar uma prateleira, ajuste esse arquivo e gere esta planilha de novo, para as abas Locais e Listas acompanharem.</t>
+          <t>Os móveis, as medidas e as gavetas de cada um ficam no próprio site, no arquivo laboratorio.js, e não nesta planilha.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>Se um móvel mudar de lugar ou ganhar uma prateleira, ajuste esse arquivo e gere esta planilha de novo, para as abas Locais e Listas acompanharem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>Os itens marcados como "Cadastrado pela foto" foram lidos das fotos do laboratório. Confira e apague a observação.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="3" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Não mude os nomes das abas nem os títulos das colunas da aba Estoque: o site procura por eles.</t>
         </is>
@@ -334,7 +341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -349,6 +356,7 @@
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -412,6 +420,11 @@
           <t>Observações</t>
         </is>
       </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -958,22 +971,35 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Termo retrátil</t>
+          <t>Garra azul de solda</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>No organizador transparente</t>
+          <t>De prender na mesa, com 3 braços flexíveis e garras jacaré</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrada em 27/10/2026, com a foto do produto. Conferir no laboratório.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>imagens/garra-azul-de-solda.jpg</t>
         </is>
       </c>
     </row>
@@ -985,7 +1011,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>P3B-1</t>
+          <t>P3B</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -995,30 +1021,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Ferramentas</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ferro de solda</t>
+          <t>Termo retrátil</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Cabo amarelo e preto</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>un</t>
+          <t>No organizador transparente</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1045,12 +1063,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ferro de solda Hikari</t>
+          <t>Ferro de solda</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Cabo branco</t>
+          <t>Cabo amarelo e preto</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -1090,12 +1108,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Suporte para ferro de solda Yaxun</t>
+          <t>Ferro de solda Hikari</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Azul, com bandeja para a esponja</t>
+          <t>Cabo branco</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -1135,12 +1153,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Alicate de corte rente Hikari</t>
+          <t>Suporte para ferro de solda Yaxun</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Cabo amarelo e preto</t>
+          <t>Azul, com bandeja para a esponja</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -1180,12 +1198,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Alicate de corte rente pequeno</t>
+          <t>Alicate de corte rente Hikari</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Cabo cinza</t>
+          <t>Cabo amarelo e preto</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1225,12 +1243,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Alicate crimpador de terminais</t>
+          <t>Alicate de corte rente pequeno</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Cabo vermelho e azul</t>
+          <t>Cabo cinza</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1270,12 +1288,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Alicate desencapador automático</t>
+          <t>Alicate crimpador de terminais</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Laranja e amarelo</t>
+          <t>Cabo vermelho e azul</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1320,7 +1338,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Vermelho e preto</t>
+          <t>Laranja e amarelo</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1360,12 +1378,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pinça antiestática</t>
+          <t>Alicate desencapador automático</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>No saquinho amarelo</t>
+          <t>Vermelho e preto</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1373,12 +1391,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Confira quantas pinças tem no saquinho.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1405,12 +1423,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Jogo de pinças antiestáticas</t>
+          <t>Pinça antiestática</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>6 pinças, pontas retas e curvas</t>
+          <t>No saquinho amarelo</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1423,7 +1441,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Confira quantas pinças tem no saquinho.</t>
         </is>
       </c>
     </row>
@@ -1445,30 +1463,30 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Estanho (fio de solda)</t>
+          <t>Jogo de pinças antiestáticas</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Carretel</t>
+          <t>6 pinças, pontas retas e curvas</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>rolo</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Parecem 2 carretéis empilhados.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1495,25 +1513,25 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Pasta de solda Cobix</t>
+          <t>Estanho (fio de solda)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Pote de 110 g</t>
+          <t>Carretel</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>rolo</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Parecem 2 carretéis empilhados.</t>
         </is>
       </c>
     </row>
@@ -1540,12 +1558,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fluxo de solda líquido</t>
+          <t>Pasta de solda Cobix</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Frasco com bico; o rótulo começa com "Res"</t>
+          <t>Pote de 110 g</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -1558,7 +1576,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Leia o rótulo para confirmar o que é.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1585,12 +1603,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Malha dessoldadora</t>
+          <t>Fluxo de solda líquido</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Carretel pequeno roxo</t>
+          <t>Frasco com bico; o rótulo começa com "Res"</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -1603,7 +1621,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Leia o rótulo para confirmar o que é.</t>
         </is>
       </c>
     </row>
@@ -1625,17 +1643,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Ferramentas</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Sugador de solda</t>
+          <t>Malha dessoldadora</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Azul</t>
+          <t>Carretel pequeno roxo</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -1675,12 +1693,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Escova pequena de limpeza</t>
+          <t>Sugador de solda</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Cerdas pretas</t>
+          <t>Azul</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -1720,12 +1738,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Manta de silicone para solda</t>
+          <t>Escova pequena de limpeza</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Azul, com divisórias</t>
+          <t>Cerdas pretas</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -1738,7 +1756,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Confira se ela fica guardada no cesto.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório.</t>
         </is>
       </c>
     </row>
@@ -1753,19 +1771,24 @@
           <t>P3B-1</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Ferramentas</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Peça preta de plástico</t>
+          <t>Manta de silicone para solda</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Retangular, com uma janela no meio</t>
+          <t>Azul, com divisórias</t>
         </is>
       </c>
       <c r="G32" t="n">
@@ -1778,7 +1801,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Não deu para saber o que é pela foto.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Confira se ela fica guardada no cesto.</t>
         </is>
       </c>
     </row>
@@ -1790,22 +1813,35 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>P3C-3</t>
+          <t>P3B-1</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Cola quente</t>
+          <t>Peça preta de plástico</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Retangular, com uma janela no meio</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+          <t>Cadastrado pela foto do cesto de solda de 27/10/2026. Conferir no laboratório. Não deu para saber o que é pela foto.</t>
         </is>
       </c>
     </row>
@@ -1817,22 +1853,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>P3C-6</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Eletrônica</t>
+          <t>P3C-3</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Conectores</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Terminais</t>
+          <t>Cola quente</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -1849,7 +1880,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>P3C-10</t>
+          <t>P3C-6</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1859,12 +1890,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Conectores</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Cabos</t>
+          <t>Terminais</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -1881,7 +1912,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>P3C-11</t>
+          <t>P3C-10</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1891,12 +1922,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Placas e controladores</t>
+          <t>Fios e cabos</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Arduino</t>
+          <t>Cabos</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -1913,7 +1944,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>P3C-12</t>
+          <t>P3C-11</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1923,12 +1954,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Placas e controladores</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Cabo USB do Arduino</t>
+          <t>Arduino</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -1945,22 +1976,22 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>P3D-1</t>
+          <t>P3C-12</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Fios e cabos</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Fita crepe</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>rolo</t>
+          <t>Cabo USB do Arduino</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -1977,27 +2008,22 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>P3D-2</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Eletrônica</t>
+          <t>P3D-1</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Protoboard</t>
+          <t>Fita crepe</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>rolo</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -2014,7 +2040,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>P3D-4</t>
+          <t>P3D-2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2024,17 +2050,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Consumíveis</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Fita isolante</t>
+          <t>Protoboard</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>rolo</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -2051,7 +2077,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>P3D-8</t>
+          <t>P3D-4</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2061,17 +2087,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Baterias</t>
+          <t>Consumíveis</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Pilhas</t>
+          <t>Fita isolante</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>rolo</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -2088,7 +2114,7 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>P3D-10</t>
+          <t>P3D-8</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2098,12 +2124,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Fios e cabos</t>
+          <t>Baterias</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Jumpers</t>
+          <t>Pilhas</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -2120,7 +2151,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>P3D-11</t>
+          <t>P3D-10</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2152,7 +2183,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>P3D-12</t>
+          <t>P3D-11</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2184,7 +2215,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>P3D-13</t>
+          <t>P3D-12</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2216,40 +2247,72 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
+          <t>P3D-13</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Eletrônica</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Fios e cabos</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Jumpers</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Pela etiqueta da caixinha, na foto de 26/10/2026. Conferir no laboratório.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Armário 3</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
           <t>P3D</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Consumíveis</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Borrifador</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Líquido transparente</t>
         </is>
       </c>
-      <c r="G46" t="n">
+      <c r="G47" t="n">
         <v>1</v>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>un</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>Cadastrado pela foto de 26/10/2026. Conferir no laboratório. Confira o que tem dentro.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1000"/>
+  <autoFilter ref="A1:M1000"/>
   <dataValidations count="5">
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha uma opção da lista. As opções ficam na aba Listas." type="list">
       <formula1>=Listas!$A$2:$A$60</formula1>

</xml_diff>